<commit_message>
docs(tracker): add model-fallback (E3 S8) + admin model-switcher (E10 S6)
Founder review before Sprint 2 surfaced two roadmap gaps in the model layer:

- E3-08.4 (Epic 3, Sprint 8): model fallback CHAINS + graceful model
  degradation. Today only KEY fallback exists (Anthropic key -> Emergent
  universal key, same model); no cross-model fallback if the model itself
  errors/times out. Builds on E3-01.2 routing + E3-01.3 telemetry.
- U10-06.1 (Epic 10, Sprint 6): admin model switcher -- runtime, DB-backed
  override of model-per-task from the admin console (no redeploy), read by
  model_for(). Deferred from Epic 3 to Epic 10 per founder.

Prompt-quality (evals track + per-domain accuracy sprints) and guardrails
(Epic 3 Sprint 8: injection, PII, cost) were already covered -- no change.

Totals: Epic 3 -> 5/36, Epic 10 -> 10/72. Program Dashboard regenerated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Admin_Console.xlsx
+++ b/docs/DecisionOS_Epic10_Admin_Console.xlsx
@@ -962,6 +962,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -1212,7 +1213,7 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1373,7 +1374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2032,6 +2033,66 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>U10-06.1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Admin console + AI model routing</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>6</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Admin model switcher -- change model-per-task at runtime</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Runtime, DB-backed override of MODEL_ROUTES per AI task from the super-admin console (no redeploy). model_for() reads an override layer first: env -&gt; DB override -&gt; MODEL_ROUTES -&gt; default. Admin picks the model per task from the MODELS catalog; the change is audited. Pairs with the AI quality dashboard (E3-10.2) so the effect of a switch is visible.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>E3-01.2</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Added 2026-08-25. Deferred from the Epic 3 model-routing discussion to Epic 10 per founder. TODAY models change only via config.py MODELS + MODEL_ROUTE_&lt;TASK&gt; env override (needs a redeploy). Sibling to U10-00.4 AI provider keys.</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Epic 10 S6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Epic 10 S3 COMPLETE (U10-03.1..7): support desk & tickets
- support_tickets collection + admin desk (routers/admin_support.py): inbox with
  status/priority/tenant filters + counts, ticket detail+thread, reply (-> pending),
  PATCH status/priority/assign. All mutations audited.
- Tenant-facing (routers/support.py): owners raise/list/reply on tickets; writes are
  naturally blocked under read-only impersonation.
- Jump-to-impersonation from a ticket (reuses S2).
- Frontend: Support desk admin tab (inbox -> detail -> reply/status/view-as-tenant).

Verified: full lifecycle (raise -> inbox -> reply -> resolve) + ruff clean. 9 new routes
-> API-parity baseline regenerated (271 -> 280 method-rows); parity green.
Tracker: Epic 10 Backlog +7 (S3 7/7), Epic 10 30/73; Master 421/605.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Admin_Console.xlsx
+++ b/docs/DecisionOS_Epic10_Admin_Console.xlsx
@@ -1111,19 +1111,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D9" t="n">
         <v>7</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1374,7 +1374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2612,7 +2612,6 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>core/security.py</t>
@@ -2921,6 +2920,422 @@
       <c r="L26" t="inlineStr">
         <is>
           <t>Epic 10 S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>U10-03.1</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Admin / Support</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Ticket model + create</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>support_tickets collection {tenant, subject, status(open/pending/resolved/closed), priority(low/normal/high/urgent), created_by(+type), assigned_admin, messages[]}. Created by admin (on a tenant's behalf) or by a tenant owner.</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>routers/admin_support.py</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Epic 10 S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>U10-03.2</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Admin / Support</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Ticket inbox (filter + counts)</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>GET /admin/tickets?status=&amp;priority=&amp;tenant_id= -&gt; newest-first list (messages omitted) + per-status counts.</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>U10-03.1</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>routers/admin_support.py</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Epic 10 S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>U10-03.3</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Admin / Support</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Ticket detail + thread</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>GET /admin/tickets/{id} -&gt; full ticket incl. message thread.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>U10-03.1</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>routers/admin_support.py</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Epic 10 S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>U10-03.4</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Admin / Support</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Reply + status/priority/assign</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>POST /admin/tickets/{id}/reply (adds admin msg, -&gt; pending) + PATCH /admin/tickets/{id} (status/priority/assigned_admin). Audited.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>U10-03.1</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>routers/admin_support.py</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Epic 10 S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>U10-03.5</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Admin / Support</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Jump to impersonation from ticket</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Ticket detail 'View as tenant' starts a read-only impersonation session for the ticket's workspace (reuses S2).</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>U10-03.3</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>frontend SupportDeskSection</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Epic 10 S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>U10-03.6</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Support (tenant)</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Tenant-facing ticket submission</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>routers/support.py: POST /api/support/tickets (owner/member raises), GET /api/support/tickets (their tickets), reply. Writes naturally blocked under read-only impersonation.</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>U10-03.1</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>routers/support.py</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Epic 10 S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>U10-03.7</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Admin portal</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Support desk tab</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Inbox with status filter + counts -&gt; ticket detail (thread, reply box, status/priority selects, view-as-tenant). SupportDeskSection.js.</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>U10-03.2</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/admin/SupportDeskSection.js</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Epic 10 S3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Epic 10 S5 COMPLETE (U10-05.1..6): observability & logs
routers/admin_observability.py -- platform reliability from recorded telemetry:
- GET /admin/observability/reliability?range=: error rate, degraded/fallback rate,
  latency p50/p95/max, breakdowns by provider (engine) + task (1h/24h/7d/30d).
- GET /admin/observability/errors: recent failed AI calls (error text PII-redacted).
- GET /admin/observability/outages: platform_alerts timeline, active-first.
Frontend: Observability tab (reliability cards + by-provider/task + errors + outage timeline).

NOTE: rate-limit is in-memory (not persisted), so fallback/degraded rate is the reliability
signal instead of stored rate-limit hits.

Verified against real telemetry (260 calls, p50 3.3s/p95 8.6s, anthropic 191/openai 69);
ruff clean. 3 new routes -> parity baseline 285 -> 288; parity green.
Tracker: Epic 10 Backlog +6 (S5 6/6), Epic 10 43/73; Master 434/605.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Admin_Console.xlsx
+++ b/docs/DecisionOS_Epic10_Admin_Console.xlsx
@@ -1177,19 +1177,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D11" t="n">
         <v>6</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -1374,7 +1374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3382,7 +3382,6 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
           <t>routers/admin_billing.py</t>
@@ -3751,6 +3750,358 @@
       <c r="L40" t="inlineStr">
         <is>
           <t>Epic 10 S4</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>U10-05.1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Admin / Observability</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>5</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>AI reliability + latency</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>GET /admin/observability/reliability?range=: error rate, degraded/fallback rate, latency p50/p95/max, breakdowns by provider (engine) + task, over 1h/24h/7d/30d.</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>routers/admin_observability.py</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Epic 10 S5</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>U10-05.2</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Admin / Observability</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>5</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Recent-errors log viewer</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>GET /admin/observability/errors: recent failed AI calls (ok=False) with task/model/engine/error(PII-redacted)/tenant/time.</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>U10-05.1</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>routers/admin_observability.py</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Epic 10 S5</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>U10-05.3</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Admin / Observability</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>5</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Provider-outage timeline</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>GET /admin/observability/outages: platform_alerts history, active-first, with resolved/active status + active count.</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>routers/admin_observability.py</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Epic 10 S5</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>U10-05.4</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Admin / Observability</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>5</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Error aggregation by task/provider</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Per-task + per-provider error + degraded counts in the reliability payload (the aggregation surface).</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>U10-05.1</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>routers/admin_observability.py</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Epic 10 S5</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>U10-05.5</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Admin / Observability</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>5</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Latency / slow-call signals</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Latency percentiles (p50/p95/max) overall + avg per provider/task from ai_calls.latency_ms. NOTE: rate-limit is in-memory (not persisted) -&gt; fallback/degraded rate is the reliability signal instead.</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>U10-05.1</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>routers/admin_observability.py</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Epic 10 S5</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>U10-05.6</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Admin portal</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>5</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Observability tab</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Reliability cards (calls / error rate / fallback / p95 latency) + by-provider/by-task tables + recent-errors viewer + outage timeline, with a range selector. ObservabilitySection.js.</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>U10-05.1</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/admin/ObservabilitySection.js</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Epic 10 S5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Epic 10: log U10-QA.1 (admin_usage aggregate coroutine bugfix)
Backlog + dashboard note the QA fix landed in 743a957 during the browser
preview walk-through of the console. Keeps the tracker aligned with the
code push (every shipped fix updates the tracker in the same series).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Admin_Console.xlsx
+++ b/docs/DecisionOS_Epic10_Admin_Console.xlsx
@@ -958,11 +958,10 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Epic 10 IN PROGRESS. S0 shipped + S1-S8 COMPLETE (Tenant 360, impersonation, support desk, billing, observability, feature-flags/config, admin RBAC+2FA, announcements). 8 new admin tabs + a tenant announcement banner; 60+ new routes; route fingerprint tracked via the committed API-parity baseline. Remaining: S9 (compliance/DPDP data ops) + S10 (admin polish, tests &amp; QA).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
+          <t>Epic 10 IN PROGRESS. S0 shipped + S1-S8 COMPLETE (Tenant 360, impersonation, support desk, billing, observability, feature-flags/config, admin RBAC+2FA, announcements). 8 new admin tabs + a tenant announcement banner; 60+ new routes; route fingerprint tracked via the committed API-parity baseline. Browser preview QA: full 16-tab walk-through green after a motor aggregate() coroutine fix in admin_usage (see backlog U10-QA.1). Remaining: S9 (compliance/DPDP data ops) + S10 (admin polish, tests &amp; QA).</t>
+        </is>
+      </c>
+    </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -1374,7 +1373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4777,7 +4776,6 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
         <is>
           <t>routers/admin_announcements.py</t>
@@ -5026,6 +5024,62 @@
       <c r="L62" t="inlineStr">
         <is>
           <t>Epic 10 S8</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>U10-QA.1</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Admin / Usage</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Bugfix</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Fix admin_usage motor aggregate() coroutine bug</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Split `db.usage_events.aggregate(...).to_list()` into `_cur = await db...aggregate(...); await _cur.to_list(N)` in both the per-provider and per-workspace queries. Under motor 3.x aggregate() returns a coroutine so chained .to_list() raised AttributeError -&gt; 500. Caught in browser QA walk-through of the Admin &gt; Usage tab; endpoint now returns 200 OK.</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>routers/admin.py (S0 admin_usage)</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Epic 10 QA fix (browser preview walk-through)</t>
         </is>
       </c>
     </row>

</xml_diff>